<commit_message>
Rebuild syllabus and Đợt 0–10 exercises on SKU1 formula of 24/09/2026
Add the 22-ingredient formula (roles, INCI corrections, allowed and
forbidden claims) to the syllabus and Đợt 0 Product Truth Sheet, align
positioning, proof, assets, hooks and evidence log in Đợt 2–10, fill
ingredient placeholders in the 30 TikTok contents, and drop the company
name from page footers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RCHR5nifryaMfRHokNNBvc
</commit_message>
<xml_diff>
--- a/DS CORPORATION/TÀI LIỆU THAM KHẢO/MARKETING ROADMAP/BAI TAP/Bo_cong_cu_Dot2-10.xlsx
+++ b/DS CORPORATION/TÀI LIỆU THAM KHẢO/MARKETING ROADMAP/BAI TAP/Bo_cong_cu_Dot2-10.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="483">
   <si>
     <t xml:space="preserve">Bộ công cụ Đợt 2–10 · Dosie's Care</t>
   </si>
@@ -754,6 +754,9 @@
     <t xml:space="preserve">Hành động</t>
   </si>
   <si>
+    <t xml:space="preserve">Cảm giác mát lạnh bạc hà + hương bưởi da xanh</t>
+  </si>
+  <si>
     <t xml:space="preserve">Monogram DS (bướm + chữ D, S)</t>
   </si>
   <si>
@@ -841,13 +844,13 @@
     <t xml:space="preserve">Ủ tóc mà sợ bết? Lỗi nằm ở bước gội, không phải ở việc ủ.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mẹo gội sạch ngay lần đầu sau khi ủ: nhũ hóa.</t>
+    <t xml:space="preserve">Mẹo gội sạch ngay lần đầu sau khi ủ: sữa gội lên tóc khô trước, nước sau.</t>
   </si>
   <si>
     <t xml:space="preserve">Ủ qua đêm có tốt hơn không? Không hẳn.</t>
   </si>
   <si>
-    <t xml:space="preserve">Kết cấu đặc và kết cấu nhẹ: thử trên mu bàn tay.</t>
+    <t xml:space="preserve">Massage thấy mát lạnh? Đó là bạc hà, không phải "thuốc".</t>
   </si>
   <si>
     <t xml:space="preserve">Lười massage 10 phút? Gắn nó vào giờ tắm.</t>
@@ -868,7 +871,7 @@
     <t xml:space="preserve">Mình ủ rồi gội đúng 1 lần: kết quả thật, không cắt.</t>
   </si>
   <si>
-    <t xml:space="preserve">Đọc cùng mình bảng thành phần chai này.</t>
+    <t xml:space="preserve">22 thành phần trong chai này, cái nào làm gì? Đọc cùng mình.</t>
   </si>
   <si>
     <t xml:space="preserve">3 bước, 15 phút, gắn vào giờ tắm.</t>
@@ -1433,6 +1436,54 @@
   </si>
   <si>
     <t xml:space="preserve">Chờ thí nghiệm backlog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bạc hà tạo cảm giác mát (menthol kích hoạt thụ thể lạnh TRPM8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">McKemy et al., Nature 2002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nghiên cứu cơ chế</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chỉ giải thích cảm giác, không phải tác dụng trên tóc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jojoba là sáp lỏng (wax ester), cùng loại lipid với một phần bã nhờn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Picardo et al., Dermato-Endocrinology 2009 (thành phần bã nhờn người)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y văn hóa sinh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giống về loại chất, không chứng minh "điều tiết bã nhờn"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tinh dầu hương thảo so với minoxidil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panahi et al., Skinmed 2015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 thử nghiệm nhỏ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**Không dùng trong marketing**: so với thuốc biến mỹ phẩm thành thuốc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tinh dầu tràm trà và gàu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Satchell et al., JAAD 2002 (dầu gội 5%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thử nghiệm lâm sàng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**Không dùng**: trị gàu là công dụng thuốc; nồng độ trong DS khác</t>
   </si>
 </sst>
 </file>
@@ -2171,7 +2222,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2179,13 +2230,13 @@
         <v>57</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>154</v>
@@ -2203,7 +2254,7 @@
         <v>55</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2211,10 +2262,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -2232,10 +2283,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -2253,10 +2304,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
@@ -2274,10 +2325,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
@@ -2295,10 +2346,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
@@ -2316,10 +2367,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
@@ -2337,10 +2388,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
@@ -2358,10 +2409,10 @@
         <v>8</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
@@ -2379,10 +2430,10 @@
         <v>9</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
@@ -2400,10 +2451,10 @@
         <v>10</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
@@ -2421,10 +2472,10 @@
         <v>11</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
@@ -2442,10 +2493,10 @@
         <v>12</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
@@ -2463,10 +2514,10 @@
         <v>13</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
@@ -2484,10 +2535,10 @@
         <v>14</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
@@ -2500,15 +2551,15 @@
       </c>
       <c r="J18" s="9"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
@@ -2526,10 +2577,10 @@
         <v>16</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
@@ -2547,10 +2598,10 @@
         <v>17</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
@@ -2568,10 +2619,10 @@
         <v>18</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
@@ -2589,10 +2640,10 @@
         <v>19</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
@@ -2610,10 +2661,10 @@
         <v>20</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
@@ -2631,10 +2682,10 @@
         <v>21</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
@@ -2652,10 +2703,10 @@
         <v>22</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
@@ -2673,10 +2724,10 @@
         <v>23</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
@@ -2694,10 +2745,10 @@
         <v>24</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
@@ -2715,10 +2766,10 @@
         <v>25</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
@@ -2736,10 +2787,10 @@
         <v>26</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
@@ -2757,10 +2808,10 @@
         <v>27</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
@@ -2778,10 +2829,10 @@
         <v>28</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
@@ -2799,10 +2850,10 @@
         <v>29</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
@@ -2820,10 +2871,10 @@
         <v>30</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
@@ -2884,56 +2935,56 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>147</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -2957,7 +3008,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -2981,7 +3032,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -3005,7 +3056,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -3029,7 +3080,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -3053,7 +3104,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -3077,7 +3128,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -3101,7 +3152,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -3125,7 +3176,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -3149,7 +3200,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -3173,7 +3224,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -3197,7 +3248,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -3221,7 +3272,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -3245,7 +3296,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -3269,7 +3320,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
@@ -3293,7 +3344,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -3317,7 +3368,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
@@ -3341,7 +3392,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
@@ -3365,7 +3416,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
@@ -3389,7 +3440,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
@@ -3413,7 +3464,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
@@ -3437,7 +3488,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -3461,7 +3512,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
@@ -3485,7 +3536,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -3509,7 +3560,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
@@ -3533,7 +3584,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -3557,7 +3608,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B31" s="9"/>
       <c r="C31" s="9"/>
@@ -3581,7 +3632,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B32" s="9"/>
       <c r="C32" s="9"/>
@@ -3605,7 +3656,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
@@ -3629,7 +3680,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -3653,7 +3704,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -3677,7 +3728,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
@@ -3701,7 +3752,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="8" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
@@ -3725,7 +3776,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="8" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B38" s="9"/>
       <c r="C38" s="9"/>
@@ -3749,7 +3800,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
@@ -3773,7 +3824,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="8" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B40" s="9"/>
       <c r="C40" s="9"/>
@@ -3797,7 +3848,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="8" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B41" s="9"/>
       <c r="C41" s="9"/>
@@ -3821,7 +3872,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="8" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B42" s="9"/>
       <c r="C42" s="9"/>
@@ -3845,7 +3896,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="8" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B43" s="9"/>
       <c r="C43" s="9"/>
@@ -3869,7 +3920,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="8" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B44" s="9"/>
       <c r="C44" s="9"/>
@@ -3932,12 +3983,12 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>167</v>
@@ -3945,21 +3996,21 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B5" s="18"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">IF(B6="Tháng 1–3",0.3,IF(B6="Tháng 4–6",0.4,0.5))</f>
@@ -3968,7 +4019,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B8" s="17" t="str">
         <f aca="false">IF(ISNUMBER(B5),B5*B7,"")</f>
@@ -3977,7 +4028,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B9" s="17" t="str">
         <f aca="false">IF(ISNUMBER(B5),B5-B8,"")</f>
@@ -3989,21 +4040,21 @@
         <v>147</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C12" s="19" t="n">
         <v>0.5</v>
@@ -4015,10 +4066,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>353</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>352</v>
       </c>
       <c r="C13" s="19" t="n">
         <v>0.3</v>
@@ -4030,10 +4081,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C14" s="19" t="n">
         <v>0.2</v>
@@ -4045,10 +4096,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C15" s="19" t="n">
         <v>0.45</v>
@@ -4060,10 +4111,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>357</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>356</v>
       </c>
       <c r="C16" s="19" t="n">
         <v>0.2</v>
@@ -4075,10 +4126,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C17" s="19" t="n">
         <v>0.2</v>
@@ -4090,10 +4141,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C18" s="19" t="n">
         <v>0.15</v>
@@ -4105,7 +4156,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C19" s="15" t="n">
         <f aca="false">SUMIF(B12:B18,"Brand",C12:C18)</f>
@@ -4169,52 +4220,52 @@
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5191,7 +5242,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5199,31 +5250,31 @@
         <v>57</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>31</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="H4" s="7" t="s">
         <v>208</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5231,10 +5282,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>8</v>
@@ -5254,7 +5305,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J5" s="9"/>
     </row>
@@ -5263,10 +5314,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>8</v>
@@ -5286,7 +5337,7 @@
         <v>17</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J6" s="9"/>
     </row>
@@ -5295,10 +5346,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>6</v>
@@ -5318,7 +5369,7 @@
         <v>11</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J7" s="9"/>
     </row>
@@ -5327,10 +5378,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D8" s="9" t="n">
         <v>7</v>
@@ -5350,7 +5401,7 @@
         <v>6</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J8" s="9"/>
     </row>
@@ -5359,10 +5410,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>6</v>
@@ -5382,7 +5433,7 @@
         <v>26</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J9" s="9"/>
     </row>
@@ -5391,10 +5442,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>7</v>
@@ -5414,7 +5465,7 @@
         <v>24</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J10" s="9"/>
     </row>
@@ -5423,10 +5474,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D11" s="9" t="n">
         <v>8</v>
@@ -5446,7 +5497,7 @@
         <v>2</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J11" s="9"/>
     </row>
@@ -5455,10 +5506,10 @@
         <v>8</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D12" s="9" t="n">
         <v>6</v>
@@ -5478,7 +5529,7 @@
         <v>17</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J12" s="9"/>
     </row>
@@ -5487,10 +5538,10 @@
         <v>9</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>7</v>
@@ -5510,7 +5561,7 @@
         <v>24</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J13" s="9"/>
     </row>
@@ -5519,10 +5570,10 @@
         <v>10</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D14" s="9" t="n">
         <v>7</v>
@@ -5542,7 +5593,7 @@
         <v>3</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J14" s="9"/>
     </row>
@@ -5551,10 +5602,10 @@
         <v>11</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D15" s="9" t="n">
         <v>6</v>
@@ -5574,7 +5625,7 @@
         <v>26</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J15" s="9"/>
     </row>
@@ -5583,10 +5634,10 @@
         <v>12</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D16" s="9" t="n">
         <v>6</v>
@@ -5606,7 +5657,7 @@
         <v>11</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J16" s="9"/>
     </row>
@@ -5615,10 +5666,10 @@
         <v>13</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D17" s="9" t="n">
         <v>5</v>
@@ -5638,7 +5689,7 @@
         <v>20</v>
       </c>
       <c r="I17" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J17" s="9"/>
     </row>
@@ -5647,10 +5698,10 @@
         <v>14</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D18" s="9" t="n">
         <v>6</v>
@@ -5670,7 +5721,7 @@
         <v>20</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J18" s="9"/>
     </row>
@@ -5679,10 +5730,10 @@
         <v>15</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D19" s="9" t="n">
         <v>7</v>
@@ -5702,7 +5753,7 @@
         <v>6</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J19" s="9"/>
     </row>
@@ -5711,10 +5762,10 @@
         <v>16</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D20" s="9" t="n">
         <v>7</v>
@@ -5734,7 +5785,7 @@
         <v>16</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J20" s="9"/>
     </row>
@@ -5743,10 +5794,10 @@
         <v>17</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D21" s="9" t="n">
         <v>5</v>
@@ -5766,7 +5817,7 @@
         <v>20</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J21" s="9"/>
     </row>
@@ -5775,10 +5826,10 @@
         <v>18</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D22" s="9" t="n">
         <v>6</v>
@@ -5798,7 +5849,7 @@
         <v>11</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J22" s="9"/>
     </row>
@@ -5807,10 +5858,10 @@
         <v>19</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>7</v>
@@ -5830,7 +5881,7 @@
         <v>3</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J23" s="9"/>
     </row>
@@ -5839,10 +5890,10 @@
         <v>20</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D24" s="9" t="n">
         <v>6</v>
@@ -5862,7 +5913,7 @@
         <v>11</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J24" s="9"/>
     </row>
@@ -5871,10 +5922,10 @@
         <v>21</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D25" s="9" t="n">
         <v>6</v>
@@ -5894,7 +5945,7 @@
         <v>20</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J25" s="9"/>
     </row>
@@ -5903,10 +5954,10 @@
         <v>22</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D26" s="9" t="n">
         <v>7</v>
@@ -5926,7 +5977,7 @@
         <v>6</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J26" s="9"/>
     </row>
@@ -5935,10 +5986,10 @@
         <v>23</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D27" s="9" t="n">
         <v>8</v>
@@ -5958,7 +6009,7 @@
         <v>17</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J27" s="9"/>
     </row>
@@ -5967,10 +6018,10 @@
         <v>24</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D28" s="9" t="n">
         <v>6</v>
@@ -5990,7 +6041,7 @@
         <v>3</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J28" s="9"/>
     </row>
@@ -5999,10 +6050,10 @@
         <v>25</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D29" s="9" t="n">
         <v>6</v>
@@ -6022,7 +6073,7 @@
         <v>6</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J29" s="9"/>
     </row>
@@ -6031,10 +6082,10 @@
         <v>26</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>6</v>
@@ -6054,7 +6105,7 @@
         <v>28</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J30" s="9"/>
     </row>
@@ -6063,10 +6114,10 @@
         <v>27</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D31" s="9" t="n">
         <v>6</v>
@@ -6086,7 +6137,7 @@
         <v>30</v>
       </c>
       <c r="I31" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J31" s="9"/>
     </row>
@@ -6098,7 +6149,7 @@
         <v>130</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D32" s="9" t="n">
         <v>7</v>
@@ -6118,7 +6169,7 @@
         <v>6</v>
       </c>
       <c r="I32" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J32" s="9"/>
     </row>
@@ -6130,7 +6181,7 @@
         <v>130</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D33" s="9" t="n">
         <v>7</v>
@@ -6150,7 +6201,7 @@
         <v>28</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J33" s="9"/>
     </row>
@@ -6159,10 +6210,10 @@
         <v>30</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D34" s="9" t="n">
         <v>6</v>
@@ -6182,7 +6233,7 @@
         <v>11</v>
       </c>
       <c r="I34" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="J34" s="9"/>
     </row>
@@ -6233,7 +6284,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6241,28 +6292,28 @@
         <v>57</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="H4" s="7" t="s">
         <v>153</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6270,16 +6321,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F5" s="9"/>
       <c r="G5" s="9"/>
@@ -6294,16 +6345,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F6" s="9"/>
       <c r="G6" s="9"/>
@@ -6318,16 +6369,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F7" s="9"/>
       <c r="G7" s="9"/>
@@ -6342,16 +6393,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F8" s="9"/>
       <c r="G8" s="9"/>
@@ -6366,16 +6417,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F9" s="9"/>
       <c r="G9" s="9"/>
@@ -6390,16 +6441,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
@@ -6414,16 +6465,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F11" s="9"/>
       <c r="G11" s="9"/>
@@ -6438,16 +6489,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="F12" s="9"/>
       <c r="G12" s="9"/>
@@ -6462,16 +6513,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="F13" s="9"/>
       <c r="G13" s="9"/>
@@ -6486,16 +6537,16 @@
         <v>10</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="F14" s="9"/>
       <c r="G14" s="9"/>
@@ -6505,14 +6556,22 @@
         <v/>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
+      <c r="B15" s="8" t="s">
+        <v>467</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>468</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>469</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>470</v>
+      </c>
       <c r="F15" s="9"/>
       <c r="G15" s="9"/>
       <c r="H15" s="25"/>
@@ -6521,14 +6580,22 @@
         <v/>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
+      <c r="B16" s="8" t="s">
+        <v>471</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>472</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>473</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>474</v>
+      </c>
       <c r="F16" s="9"/>
       <c r="G16" s="9"/>
       <c r="H16" s="25"/>
@@ -6537,14 +6604,22 @@
         <v/>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
+      <c r="B17" s="8" t="s">
+        <v>475</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>476</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>477</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>478</v>
+      </c>
       <c r="F17" s="9"/>
       <c r="G17" s="9"/>
       <c r="H17" s="25"/>
@@ -6553,14 +6628,22 @@
         <v/>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
+      <c r="B18" s="8" t="s">
+        <v>479</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>480</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>481</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>482</v>
+      </c>
       <c r="F18" s="9"/>
       <c r="G18" s="9"/>
       <c r="H18" s="25"/>
@@ -12358,7 +12441,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
@@ -12407,7 +12490,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
         <v>239</v>
       </c>
@@ -12455,7 +12538,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
         <v>241</v>
       </c>
@@ -12479,7 +12562,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
         <v>242</v>
       </c>
@@ -12572,6 +12655,30 @@
       </c>
       <c r="H11" s="8" t="str">
         <f aca="false">IF(G11="Dùng ngay","Lặp lại ở mọi điểm chạm",IF(G11="Đầu tư thêm","Lặp lại nhiều hơn để tăng fame",IF(G11="Dễ nhầm, cẩn trọng","Ghép với tài sản riêng của DS",IF(G11="","","Không đầu tư"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="15" t="str">
+        <f aca="false">IF(AND(ISNUMBER(B12),B12&gt;0),C12/B12,"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="15" t="str">
+        <f aca="false">IF(AND(ISNUMBER(C12),C12+D12&gt;0),C12/(C12+D12),"")</f>
+        <v/>
+      </c>
+      <c r="G12" s="8" t="str">
+        <f aca="false">IF(E12="","",IF(AND(E12&gt;=0.5,F12&gt;=0.5),"Dùng ngay",IF(F12&gt;=0.5,"Đầu tư thêm",IF(E12&gt;=0.5,"Dễ nhầm, cẩn trọng","Bỏ/thay"))))</f>
+        <v/>
+      </c>
+      <c r="H12" s="8" t="str">
+        <f aca="false">IF(G12="Dùng ngay","Lặp lại ở mọi điểm chạm",IF(G12="Đầu tư thêm","Lặp lại nhiều hơn để tăng fame",IF(G12="Dễ nhầm, cẩn trọng","Ghép với tài sản riêng của DS",IF(G12="","","Không đầu tư"))))</f>
         <v/>
       </c>
     </row>

</xml_diff>